<commit_message>
Team edits: review workbooks without the unused time column, instructions sheet for every reviewer, blind-scoring comments removed, NZ supplement report table formatting; ignore Office lock files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/eval/human_blind_scoring/rater_MengshuaiFeng.xlsx
+++ b/data/eval/human_blind_scoring/rater_MengshuaiFeng.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23040" windowHeight="9060" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23040" windowHeight="9060" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scoring" sheetId="1" state="visible" r:id="rId1"/>
@@ -188,12 +188,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -529,7 +541,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
@@ -553,16 +565,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
@@ -571,99 +583,100 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
@@ -672,7 +685,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1234,12 +1246,12 @@
   <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="8" customWidth="1" style="7" min="1" max="1"/>
-    <col width="40" customWidth="1" style="7" min="2" max="2"/>
-    <col width="55" customWidth="1" style="7" min="3" max="3"/>
-    <col width="40" customWidth="1" style="7" min="4" max="4"/>
-    <col width="30" customWidth="1" style="7" min="5" max="5"/>
-    <col width="71" customWidth="1" style="7" min="6" max="6"/>
+    <col width="8" customWidth="1" style="1" min="1" max="1"/>
+    <col width="40" customWidth="1" style="1" min="2" max="2"/>
+    <col width="55" customWidth="1" style="1" min="3" max="3"/>
+    <col width="40" customWidth="1" style="1" min="4" max="4"/>
+    <col width="30" customWidth="1" style="1" min="5" max="5"/>
+    <col width="71" customWidth="1" style="1" min="6" max="6"/>
     <col width="18.5555555555556" customWidth="1" style="3" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1274,29 +1286,29 @@
           <t>answer_to_score</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>human_score_0_4</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="165.6" customHeight="1" s="7">
-      <c r="A2" s="5" t="inlineStr">
+    <row r="2" ht="165.6" customHeight="1" s="1">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>H032</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. Does mating disruption work for codling moth in apple orchards?</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>New Zealand evidence says it works when combined with some insecticides. In 14 Hawke's Bay orchards, mating disruption cut seasonal trap catch by 70% and reduced insecticide applications (from 5.9 per season to 2.3–3.7), and larval incidence in fruit averaged about 0.01%, lower than insecticide-only orchards; damage rose when growers relied more on short-residual codling moth granulosis virus. It reduced but did not eliminate risk for nil-tolerance markets, so 3–4 sprays were still used. WSU adds that small or non-isolated orchards and high populations reduce reliability. This is evidence from specific orchards and seasons; mating disruption supplements rather than replaces other management.</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>• yes, in NZ (Hawke's Bay) trials with supplementary insecticides
 • trap catch down ~70%, fewer sprays, very low fruit infestation
@@ -1304,39 +1316,39 @@
 • small/high-pressure orchards less reliable</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>• claims mating disruption alone eliminates codling moth
 • says it has not been tested in New Zealand</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Yes, according to New Zealand research in Hawke’s Bay apple orchards. In 14 orchards, seasonal pheromone trap catch fell from 40.1 codling moths/trap before mating disruption to 11.7/trap over the following five seasons (2006–2012), and larval incidence in fruit averaged 0.01%, lower than insecticide-only orchards. Mating disruption with 3–4 insecticide sprays controlled codling moth to the standard needed; it reduced insecticide use and larval risk but did not completely eliminate risk for markets with nil tolerance, so growers must balance residual and non-residual insecticides.
 Note: this is research evidence from New Zealand, not a general grower prescription; check local labels and adviser guidance.</t>
         </is>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="G2" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="3" ht="317.4" customHeight="1" s="7">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="3" ht="317.4" customHeight="1" s="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>H046</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. How should I prune out European canker in my orchard?</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>New Zealand guidance: remove all visible cankers during winter pruning; because infected wood can extend beyond the visible canker, cut at least 300 mm below the lowest canker; scraping may not remove all infection; do not prune in rain; sometimes a whole limb or tree must go. Sterilise pruning tools between trees if infection is evident, and remove and burn infected material. Infection can occur all year wherever wounds exist; a New Zealand study found pruning cuts very susceptible and fruit picking and thinning wounds the most important natural entry sites, so inspect spurs (wilting leaves next to picking wounds can signal infection).</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>• remove all visible cankers in winter pruning
 • cut at least 300 mm below the lowest canker; don't prune in rain
@@ -1344,13 +1356,13 @@
 • wounds (pruning, picking, thinning, leaf scars) are infection sites; infection year-round</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>• recommends scraping cankers as sufficient
 • recommends pruning during rain</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>In New Zealand, prune out European canker (Neonectria ditissima) as follows, per the undated New Zealand HortInfo guidance:
 - Remove all visible cankers during winter pruning — this is described as essential.
@@ -1363,27 +1375,27 @@
 Note that this source covers cultural sanitation/pruning only and excludes chemical rates and registrations; check local labels and advisers for any chemical options. The California guidance (prune and burn early in summer, plus fall fungicide sprays) and the Pacific Northwest fire blight guidance are from different regions and/or diseases and should not be substituted for New Zealand European canker advice.</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="303.6" customHeight="1" s="7">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="4" ht="303.6" customHeight="1" s="1">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>H042</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Some leaves and young apples have dark olive-green, velvety spots, and some fruit are cracking. What is this and what should I do?</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>This is apple scab (Venturia inaequalis): velvety olive-green to black spots on leaves and fruit; fruit spots become scab-like and corky, and fruit may crack and become misshapen; badly infected leaves can yellow and drop. The fungus overwinters in fallen infected leaves, and spring rains release spores that infect young leaves and fruit. Management aims to prevent primary spring infections: reduce leaf litter (shred with a flail mower or remove it; urea on leaves before or after leaf fall speeds decomposition), prune for air movement and drying, and apply protective fungicides with exact timing and full coverage during wet periods from green tip.</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>• identifies apple scab
 • olive-green to black velvety spots; fruit spots become scabby/corky and can crack
@@ -1391,13 +1403,13 @@
 • reduce leaf litter, prune for drying, timed protective fungicides in wet periods</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>• diagnoses powdery mildew or sooty blotch
 • recommends only summer treatment and ignores primary spring infection</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Based on the symptoms described (dark olive-green, velvety spots on leaves and young fruit, along with fruit cracking), the disease is **apple scab**,. 
 **What you should do:**
@@ -1409,27 +1421,27 @@
 *Disclaimer: Pesticide products, rates, and timings mentioned in historical sources are not current recommendations or proof of local authorization. Always check local product labels and consult local advisers before applying treatments.*</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="345" customHeight="1" s="7">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="345" customHeight="1" s="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>H011</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Some branches have sunken cankers with rings around buds and leaf scars, and the bark is flaky in the centre. What is it?</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>This fits European canker (Neonectria ditissima): it starts as small dark sunken areas around buds, leaf scars or wounds, which develop concentric rings of cracking with swelling of the stem above and below, a dry flaky centre and staining of the wood beneath; white spores form in the cracks in humid weather and dark red fruiting bodies in autumn and winter. Flaky bark alone is not unique to this disease. The fungus enters through leaf scars, growth cracks and wounds, and cankers kill branches; infected wood should be pruned out well below the canker and destroyed.</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>• identifies European canker
 • sunken areas at buds/leaf scars with concentric rings; white spores or red fruiting bodies
@@ -1437,13 +1449,13 @@
 • prune out infected wood below the canker and destroy it</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>• diagnoses fire blight without considering the ring pattern
 • says the canker will heal by itself</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>These symptoms on apple most strongly suggest apple canker caused by Neonectria ditissima (European canker). Sunken cankers with concentric rings of callus around buds and leaf scars, and bark that cracks and flakes in the centre, are classic signs of this disease.
 Other possibilities to consider include Nectria or Cytospora canker, frost or winter injury, and Phytophthora or Diplodia damage. Some of these look similar, so confirmation is worth doing.
@@ -1455,27 +1467,27 @@
 If you tell me your region, cultivar and the time of year, I can help narrow the diagnosis further.</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="220.8" customHeight="1" s="7">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" ht="220.8" customHeight="1" s="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>H018</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>My apple leaves have winding or blotchy mines inside them. What is causing this and does it need treatment?</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>These are leafminer larvae feeding inside the leaf: early (sap-feeding) larvae make snake-like mines visible from the underside, later tissue-feeding larvae make tent-like blotch mines and the upper leaf surface looks light and spotted. Low populations occur in most orchards and are usually kept down by parasitic wasps; they become pests mainly when broad-spectrum sprays disrupt these parasites. Treatment depends on mine counts and parasitism: UC IPM treats only when leaves average more than five mines per leaf, or when parasitism is low; WSU found no fruit impact below about two tissue-feeding mines per leaf in the second generation. Penn State notes apple leafminer has not caused economic injury.</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>• identifies leafminer mines
 • usually controlled by parasitoids; outbreaks follow broad-spectrum sprays
@@ -1483,40 +1495,40 @@
 • often no treatment needed</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>• recommends routine spraying for any mines
 • identifies the damage as a disease</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Based on the evidence, the winding-to-blotch mines on the upper leaf surface are consistent with **apple leafminer**. The larvae make a winding linear mine that widens into a blotch mine on the upper leaf surface; frass ejected through holes in the lower epidermis often hangs in threads, and leaf portions beyond the mine may become chlorotic. Pupation occurs outside the mine, often on another leaf suspended in a silken "hammock". Infestations mostly occur on succulent shoots and sprouts.
 **Treatment:** The Pennsylvania source states this leafminer "does not appear to be economically damaging". So based on that source, treatment does not appear to be warranted. Note this is region-specific guidance (Pennsylvania) and doesn't establish status elsewhere.
 Separately, if you see irregular brown blotches rather than mines, that could be necrotic leaf blotch (a physiological disorder, fruit unaffected) or Glomerella leaf spot (fungal, with purple spots and concentric rings) — these are distinct from mines and require different approaches. The distinction matters because control strategies differ.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="317.4" customHeight="1" s="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="317.4" customHeight="1" s="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>H017</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>My apples have small red-purple rings around tiny spots, and the bark has tiny grey crusty scales. What is it and what should I do?</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>This is San Jose scale: each scale settling on fruit causes a reddish purple ring or red spot, often with a slight depression; on the bark the scales are tiny, grey to black covers. Heavy infestations weaken trees, kill twigs and limbs, and can kill young trees; infested fruit is unmarketable. Dormant-season treatment is the key control (UC IPM: oil sprays work best on the overwintering black-cap stage); crawler sprays timed by degree-days after male flight or crawler emergence are the other effective window. Natural enemies help when not disrupted by insecticides, and infested trees should be checked during pruning.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>• identifies San Jose scale
 • red/purple spots or rings on fruit; grey scale covers on bark
@@ -1524,13 +1536,13 @@
 • dormant oil (and crawler sprays timed by degree-days) as key control</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>• diagnoses a fungal fruit spot
 • recommends only foliar fungicides</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Based on the symptoms described, the issue is **San Jose scale**,. Feeding by the insect causes red spots—which fade to light red or pink as the fruit grows—around the scales on the fruit. On the tree, scale populations build up and encrust limbs and bark.
 ### Management and Control
@@ -1542,27 +1554,27 @@
 *Note: Pesticide products, rates, and application timings mentioned in historical sources are not current recommendations or proof of local registration. Always check local labels and consult a local agricultural adviser before applying treatments,.*</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="317.4" customHeight="1" s="7">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="8" ht="317.4" customHeight="1" s="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>H003</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Some leaves and young apples have dark olive-green, velvety spots, and some fruit are cracking. What is this and what should I do?</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>This is apple scab (Venturia inaequalis): velvety olive-green to black spots on leaves and fruit; fruit spots become scab-like and corky, and fruit may crack and become misshapen; badly infected leaves can yellow and drop. The fungus overwinters in fallen infected leaves, and spring rains release spores that infect young leaves and fruit. Management aims to prevent primary spring infections: reduce leaf litter (shred with a flail mower or remove it; urea on leaves before or after leaf fall speeds decomposition), prune for air movement and drying, and apply protective fungicides with exact timing and full coverage during wet periods from green tip.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>• identifies apple scab
 • olive-green to black velvety spots; fruit spots become scabby/corky and can crack
@@ -1570,13 +1582,13 @@
 • reduce leaf litter, prune for drying, timed protective fungicides in wet periods</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>• diagnoses powdery mildew or sooty blotch
 • recommends only summer treatment and ignores primary spring infection</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>This description most closely matches **apple scab**. Velvety dark olive-to-black spots on leaves and fruit are its initial symptoms, and the spots on fruit become scab-like with age and tissues may become misshapen. Fruit lesions develop a blistered or "scabby" appearance and can crack and cause deformities or uneven growth. Leaves may distort, pucker, yellow and drop early.
 Cracking alone is not diagnostic, so confirm the diagnosis with local extension or plant-health advisers, because the evidence here does not rule out other causes.
@@ -1588,27 +1600,27 @@
 The sources do not give specific fungicide products, rates or timings for your location. Check current labels and consult your local extension service or adviser before applying any treatment, as the cited guidance is from California and other US sources and may not reflect your region's registrations or timing.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="409.5" customHeight="1" s="7">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="409.5" customHeight="1" s="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>H036</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>I'm in Hawke's Bay, New Zealand. When is the fire blight risk highest and how do I know when to act?</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>New Zealand guidance says outbreaks occur at blossom when temperatures exceed 16°C, with the key infection period around flowering. A Hawke's Bay, Nelson and Waikato study (1993–1995, MARYBLYT model on Royal Gala) found few mid-bloom infection events; most predicted events were near the end of flowering or after petal fall, so secondary blooms (common on Royal Gala and Braeburn) are the main risk and early-bloom streptomycin sprays were often not aligned with infection periods. Use a risk model with weather data (a fire blight model is available through Pipfruit NZ) together with open flowers, inoculum and orchard history, and keep monitoring and removing strikes.</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>• risk is highest during blossom when temperatures exceed about 16°C
 • most infection events occur in late bloom/after petal fall; secondary blooms are at risk
@@ -1616,13 +1628,13 @@
 • monitor and remove strikes</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>• recommends routine early-bloom sprays regardless of risk
 • presents US temperature thresholds as NZ guidance</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Based on research and technical guidance for New Zealand (specifically including Hawke's Bay):
 **When the risk is highest:**
@@ -1640,27 +1652,27 @@
 * **Inspect regularly:** Inspect the orchard frequently throughout the growing season, especially from blossom to mid-summer.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="331.2" customHeight="1" s="7">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="10" ht="331.2" customHeight="1" s="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>H033</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>How do I put out pheromone dispensers to control codling moth?</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Hang hand-applied dispensers in the upper third of the canopy shortly before the first moth emergence (UC IPM uses historical biofix dates; early to avoid late mating), and reapply according to the product's life if it will not last through the season. Puffers go inside edge trees or outside second-row trees at about 20 units per quarter mile. Mating disruption works best in large, uniform, square blocks (not under about 3–5 acres per UC IPM; WSU notes small orchards under 10 acres or near pest sources may not get reliable control). In the first year or with moderate to high populations, supplementary insecticides are usually needed; keep monitoring traps (high-load lures) and fruit. Dispenser rates and placement follow the product label and local registration; the UC IPM figures are not universal.</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>• place dispensers in upper canopy before first moth flight
 • best in large uniform blocks; small/isolated issues
@@ -1668,13 +1680,13 @@
 • keep monitoring with traps and fruit checks</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>• says pheromones kill moths
 • recommends mating disruption alone for high populations</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>For codling moth in California apples, pheromone products can be hand-applied dispensers or aerosol canisters (puffers); sprayable pheromones are available but not currently recommended for pome fruit orchards because of very short residual.
 **Timing:** Using historical biofix dates, hang all pheromone products shortly before first moth emergence, in early March to early April. Early placement is important to disrupt mating of overwintering moths as soon as they emerge; a late application will require a supplemental spray treatment. Reapply dispensers per manufacturer guidelines if residual will not last through harvest or the end of the last generation.
@@ -1685,27 +1697,27 @@
 These are historical California source details, not current label rates or local recommendations; check local labels and advisers.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="248.4" customHeight="1" s="7">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="248.4" customHeight="1" s="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>H035</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Which fungicides should I worry about losing effectiveness against powdery mildew?</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>The single-site groups are the concern: DMIs (FRAC 3), QoIs (FRAC 11) and SDHIs (FRAC 7) are the main registered classes for mildew besides multisite sulfur and carbonates. A New York survey (2021–2022, abstract excerpt) screened orchard populations for resistance mutations in these three groups; at that time growers had not reported control failures, though disease incidence had increased. A New Zealand study notes DMIs act at a single site and have high resistance potential, whereas oils have multiple modes of action and low resistance risk. The survey's actual results are not included in the corpus. Resistance status and registered products differ by region; single-site fungicides are at risk, not shown to have failed everywhere.</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>• names single-site groups at risk: DMI (FRAC 3), QoI (FRAC 11), SDHI (FRAC 7)
 • no control failures reported at survey time (NY)
@@ -1713,13 +1725,13 @@
 • notes the resistance status is uncertain and should be monitored, not assumed</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>• claims widespread confirmed resistance
 • recommends repeated use of a single fungicide group</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Based on the provided evidence, the specific fungicides and chemical groups with identified resistance risks or strategy considerations for apple powdery mildew include:
 * **SDHI fungicides (FRAC Group 7):** In central Washington, using SDHI fungicides early in the season should be limited to prevent resistance development in other fungal pathogens (such as *Botrytis cinerea* and preharvest/storage rots) where these Group 7 fungicides have better activity.
@@ -1728,27 +1740,27 @@
 *Note: Pesticide products, chemical groups, and usage strategies represent historical technical guidance and vary by region and environmental conditions. Check local product labels and advisers for current registration and recommendations,.*</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="12" ht="400.2" customHeight="1" s="7">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="12" ht="400.2" customHeight="1" s="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>H037</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>My apples look fine on the outside, but when I cut them the core has mould. What is this?</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>This is moldy core: fungal growth inside the seed cavity without penetrating the flesh, usually with no external symptoms (infected fruit may colour and drop early). If the fungus enters the flesh around the core it becomes core rot (dry, corky rot; or a wet rot that develops in storage). The fungi colonise flowers and enter through an open calyx, so cultivars with an open sinus such as Delicious and Idared are most susceptible; wet weather at bloom favours it. Fungicides at bloom give mixed results; pruning and training for fast drying helps, and over-mature fruit should not be stored.</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>• identifies moldy core (core rot if flesh affected)
 • no external symptoms; enters via open calyx from flowers
@@ -1756,13 +1768,13 @@
 • pruning for drying; fungicides mixed; don't store over-mature fruit</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>• attributes it to codling moth
 • says it spreads from fruit to fruit in storage as the main mechanism</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>This sounds like **moldy core**, based on the symptoms described in the evidence. Moldy core is characterized by fungal mycelium growing within the locules (the seed cavity) without penetrating the flesh, and it typically isn't noticed until the fruit is cut open. External symptoms are rare, though infected fruit may color and fall prematurely.
 Key points:
@@ -1777,27 +1789,27 @@
 The evidence does not specify which fungal species is involved in your fruit, nor does it give current fungicide recommendations. For identification and any treatment decisions, consult your local extension service or a plant pathology advisor, and check current local labels for any product.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="13" ht="220.8" customHeight="1" s="7">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="13" ht="220.8" customHeight="1" s="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>H005</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand and have lightbrown apple moth caterpillars in my apples. What should I spray?</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>The corpus has no reviewed New Zealand guidance on which insecticides to use against lightbrown apple moth, so specific products and timings cannot be given. It does contain New Zealand evidence on a non-insecticide option: in 12 Hawke's Bay orchards (2009–2011), three-species leafroller mating disruption (600 dispensers/ha) with one insecticide in early November and threshold-based follow-up cut male trap catch by up to 98% and reduced insecticide use, with acceptably low damage; it was less effective against lightbrown apple moth in Nelson, where activity is higher. Overseas leafroller sampling advice exists but is not New Zealand-specific. New Zealand resistance-management guidance for leafrollers (NZPPS, 2024) gives general spray practice without naming products: monitor with pheromone traps to time sprays, calibrate sprayers for good coverage, target the right pest stage and rotate modes of action if control fails; growers should check locally registered labels and advisers.</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>• does not present specific insecticide products or timing as established NZ advice
 • leafroller mating disruption can cut trap catch and reduce insecticide sprays (NZ Hawke's Bay trials)
@@ -1805,40 +1817,40 @@
 • does not invent products or rates</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>• names specific insecticides or rates as NZ recommendations
 • says nothing is known about controlling it in New Zealand</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Based on the provided evidence, there are no spray recommendations for managing lightbrown apple moth caterpillars in New Zealand. 
 The only available New Zealand evidence discusses experimental leafroller mating disruption dispensers tested in 2009–2011 in Hawke's Bay. It does not provide chemical or spray prescriptions. The available spray recommendations are strictly for other leafrollers or pests located in the United States,,. 
 Please check with local New Zealand agricultural advisers and consult local product labels for current authorized treatments in your region.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14" ht="400.2" customHeight="1" s="7">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="14" ht="400.2" customHeight="1" s="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>H040</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Some leaves and young apples have dark olive-green, velvety spots, and some fruit are cracking. What is this and what should I do?</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>This is apple scab (Venturia inaequalis): velvety olive-green to black spots on leaves and fruit; fruit spots become scab-like and corky, and fruit may crack and become misshapen; badly infected leaves can yellow and drop. The fungus overwinters in fallen infected leaves, and spring rains release spores that infect young leaves and fruit. Management aims to prevent primary spring infections: reduce leaf litter (shred with a flail mower or remove it; urea on leaves before or after leaf fall speeds decomposition), prune for air movement and drying, and apply protective fungicides with exact timing and full coverage during wet periods from green tip.</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>• identifies apple scab
 • olive-green to black velvety spots; fruit spots become scabby/corky and can crack
@@ -1846,13 +1858,13 @@
 • reduce leaf litter, prune for drying, timed protective fungicides in wet periods</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>• diagnoses powdery mildew or sooty blotch
 • recommends only summer treatment and ignores primary spring infection</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>This description strongly suggests **apple scab** (*Venturia inaequalis*). The dark olive-green, velvety spots on leaves and young fruit are characteristic of scab; affected fruit can become distorted and crack, especially as they grow and the skin lesions become corky.
 There are important uncertainties to check, though: the same symptom could also fit other causes (e.g. sooty blotch/flyspeck, which is more superficial, or spray damage/other fungal spots), and cracking can have several causes. Confirming the diagnosis matters before treating.
@@ -1865,27 +1877,27 @@
 I can't confirm the diagnosis from a description alone, and I'm not supplying specific products or rates because those depend on your country's registrations and current local advice. If you tell me your region and the cultivar, I can note what's generally relevant — but local labels and advisers should govern any treatment.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="15" ht="234.6" customHeight="1" s="7">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="234.6" customHeight="1" s="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>H030</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Inside my apples there are brown winding trails and the flesh is breaking down, and the skin has small dimples. What is it?</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>This fits apple maggot (the 'railroad worm'): females lay eggs singly under the skin, causing dimpling, and the maggots tunnel through the flesh leaving brown trails; bacteria associated with the maggots make the fruit rot internally. This differs from codling moth, whose larva tunnels to the core and pushes frass out of an entry hole. Apple maggot is controlled by targeting the adult flies before egg laying, timed with traps, and by removing abandoned apple trees and dropped fruit nearby.</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>• identifies apple maggot
 • egg-laying dimples and brown winding tunnels; internal rot
@@ -1893,13 +1905,13 @@
 • control targets adults before egg laying; remove abandoned hosts and dropped fruit</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>• identifies codling moth as the cause
 • recommends targeting larvae inside fruit</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Based on the symptoms—brown winding trails through the flesh, internal tissue breakdown, and small dimples on the skin—the most likely cause is damage from the **apple maggot** (*Rhagoletis pomonella*), often referred to as the "railroad worm." 
 * **The mechanism:** The adult fly lays eggs under the skin (causing the dimples or pitted spots), and the hatching larvae tunnel through the fruit, leaving brown, winding tracks. Bacteria introduced by the larvae then cause the surrounding flesh to rot and break down.
@@ -1908,27 +1920,27 @@
 Because pest activity varies by region, check with your local agricultural extension service or expert to confirm the diagnosis and review currently authorized control methods for your area.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="16" ht="262.2" customHeight="1" s="7">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="16" ht="262.2" customHeight="1" s="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>H053</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>My apples look fine on the outside, but when I cut them the core has mould. What is this?</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>This is moldy core: fungal growth inside the seed cavity without penetrating the flesh, usually with no external symptoms (infected fruit may colour and drop early). If the fungus enters the flesh around the core it becomes core rot (dry, corky rot; or a wet rot that develops in storage). The fungi colonise flowers and enter through an open calyx, so cultivars with an open sinus such as Delicious and Idared are most susceptible; wet weather at bloom favours it. Fungicides at bloom give mixed results; pruning and training for fast drying helps, and over-mature fruit should not be stored.</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>• identifies moldy core (core rot if flesh affected)
 • no external symptoms; enters via open calyx from flowers
@@ -1936,13 +1948,13 @@
 • pruning for drying; fungicides mixed; don't store over-mature fruit</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>• attributes it to codling moth
 • says it spreads from fruit to fruit in storage as the main mechanism</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>This issue is commonly known as **core rot** (or **mouldy core**). 
 It occurs when fungi (most frequently *Alternaria*, *Cladosporium*, *Fusarium*, or *Botrytis* species) enter the apple's calyx (the blossom end) while the fruit is opening or developing. The fungus grows inside the open calyx tube into the seed cavity, creating mould in the core while leaving the outer skin and flesh appearing completely healthy.
@@ -1953,27 +1965,27 @@
 *Note: Management strategies depend on your specific location and local regulations. Always check local crop protection labels and consult local agricultural advisers before applying any treatments.*</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="17" ht="331.2" customHeight="1" s="7">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="17" ht="331.2" customHeight="1" s="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>H044</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>How do I know if my apple trees have woolly apple aphid on the roots?</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Root colonies are the most damaging and are found by looking at the roots and the crown just above them: roots develop large abnormal swellings (galls) and many short fibrous roots, and colonies with shorter whitish wax may be visible on roots and underground parts of the trunk. Above ground, infested trees may have yellowish foliage and young trees uproot easily. The aphid overwinters as nymphs on roots, which move up the trunk in spring and summer to start above-ground colonies.</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>• inspect roots and crown for galls/swellings and waxy colonies
 • signs: abnormal root swellings, fibrous roots, yellowish foliage, easily uprooted young trees
@@ -1981,12 +1993,12 @@
 • overwinters on roots and moves up the trunk</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>• says woolly apple aphid only lives on branches</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>You can't reliably tell from above-ground symptoms alone. According to the Pacific Northwest source, aerial (above-ground) infestations are not a true indication of root infestations—trees can have aerial colonies all season without their roots becoming infested. The Pennsylvania source likewise notes that the underground forms are more damaging while above-ground forms cause little damage, especially on larger trees.
 What the evidence does describe:
@@ -1996,27 +2008,27 @@
 The evidence does not provide a specific scouting or root-inspection protocol (e.g., digging and examining roots) for confirming root infestation—that detail is missing from these sources. For a definitive diagnosis you would need to inspect the root system/crown directly, ideally with local extension or advisory support.</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="18" ht="358.8" customHeight="1" s="7">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="18" ht="358.8" customHeight="1" s="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>H023</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>New apple trees I planted where an old orchard used to be are growing poorly and look stunted. What is wrong?</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>This is typical of apple replant disease: shortly after planting the block grows unevenly with stunting and short internodes, and roots are discoloured with dead tips and reduced mass; some young trees die. It is mainly caused by a soil pathogen complex (fungi such as Rhizoctonia and Ilyonectria, oomycetes such as Pythium and Phytophthora, and lesion nematodes) built up by previous tree crops. WSU recommends tolerant rootstocks as the most important control (Geneva rootstocks are generally tolerant, Malling and Malling-Merton susceptible), planting in the old grass alleys, avoiding soil saturation, using nematode-free trees, and, where used, soil fumigation or a rotation of five years or more.</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>• identifies apple replant disease
 • symptoms: uneven stunted growth, damaged roots
@@ -2024,13 +2036,13 @@
 • tolerant rootstocks (Geneva) and planting in old grass alleys</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>• blames only fertiliser shortage
 • recommends replanting the same rootstock in the same holes</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>The evidence points most directly to apple replant disease, though the supplied sources do not confirm the cause in your orchard.
 - Replant disease symptoms appear shortly after planting new trees and include uneven growth across the block, stunting, and shortened internodes. When trees are uprooted, discolored roots, root tip necrosis, and reduced root biomass can be seen. Young trees may die within the first year, and many survivors have reduced fruit production and quality. This source is from Pacific Northwest (WSU/USDA-ARS) guidance, with no established date.
@@ -2041,27 +2053,27 @@
 The evidence does not include root examination methods, soil testing, or sources on replant management options such as fumigation or rootstock choice. To confirm the cause, you would need to dig up affected trees and inspect roots for the symptoms above, and check the site for root galls or weevil and aphid activity. Consult your local extension service for diagnosis and management advice applicable to your region and current pesticide labels.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="19" ht="289.8" customHeight="1" s="7">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="19" ht="289.8" customHeight="1" s="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>H006</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>It has been a very hot, dry, dusty summer and my apple leaves are bronzing with lots of tiny mites. Why is this happening and what can I change?</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Hot, dry weather favours webspinning spider mites: they reproduce rapidly, peaking in July–August, and are most abundant in dusty and water-stressed parts of the orchard. (Apple rust mite also changes with heat: in hot, dry climates it peaks in early summer and autumn with a midsummer decline.) Cultural changes from UC IPM: keep a grass cover crop and use sprinkler irrigation to reduce dust, irrigate adequately to avoid water stress, and don't mow the cover too short or let it dry out, or mites move into trees. Monitor mites and predators and treat only above thresholds with materials least disruptive to biological control.</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>• hot dry dusty conditions and water stress favour spider mites
 • reduce dust and water stress (cover crop, irrigation)
@@ -2069,13 +2081,13 @@
 • monitor with predators; selective treatment only if needed</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>• attributes bronzing to a fungal disease
 • recommends broad-spectrum sprays as first step</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Based on the provided sources, the symptoms you are observing and your management options depend on the specific mite species present:
 ### Reasons for Leaf Bronzing and High Mite Populations
@@ -2086,27 +2098,27 @@
 *Note on pesticide usage:* Check local product labels and consult local agricultural advisers before applying any pesticide products, rates, or timings, as local authorizations vary,.</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="20" ht="124.2" customHeight="1" s="7">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="20" ht="124.2" customHeight="1" s="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>H054</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Some branches have sunken cankers with rings around buds and leaf scars, and the bark is flaky in the centre. What is it?</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>This fits European canker (Neonectria ditissima): it starts as small dark sunken areas around buds, leaf scars or wounds, which develop concentric rings of cracking with swelling of the stem above and below, a dry flaky centre and staining of the wood beneath; white spores form in the cracks in humid weather and dark red fruiting bodies in autumn and winter. Flaky bark alone is not unique to this disease. The fungus enters through leaf scars, growth cracks and wounds, and cankers kill branches; infected wood should be pruned out well below the canker and destroyed.</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>• identifies European canker
 • sunken areas at buds/leaf scars with concentric rings; white spores or red fruiting bodies
@@ -2114,39 +2126,39 @@
 • prune out infected wood below the canker and destroy it</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>• diagnoses fire blight without considering the ring pattern
 • says the canker will heal by itself</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Based on technical guidance from New Zealand, these symptoms describe **European canker**. 
 The initial symptoms of European canker appear as small, sunken areas around a bud, leaf scar, or at the base of a small dead shoot or open wound, where concentric rings begin to form and expand outward. As the disease progresses over time, the centre of the infected area dries out and becomes flaky.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="21" ht="386.4" customHeight="1" s="7">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="21" ht="386.4" customHeight="1" s="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>H027</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>When should I spray blossoms to protect against fire blight?</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Blossom sprays are only needed when infection risk is high: risk exists whenever flowers are open, the weather is warm and wetting occurs. Use a risk model to decide (e.g. Cougar Blight via the WSU Decision Aid System, Maryblyt, or the degree-hour models used in California); WSU advises applying antibiotics within the 24 hours before flower wetting after warm weather and repeating every 2–3 days during high risk, rotating modes of action, and protecting secondary blooms for about three weeks after petal fall. Most sprays protect only flowers already open. Removing cankers and strikes remains essential. Product choice and timing depend on locally registered labels, the local risk model and resistance management; one region's thresholds do not apply everywhere.</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>• spray only during high-risk periods (open flowers, warmth, wetting)
 • use a risk model to time sprays
@@ -2154,13 +2166,13 @@
 • protect secondary blooms; sanitation remains essential</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>• recommends calendar sprays throughout the season
 • states antibiotics cure existing infections</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Spray timing for blossom protection depends on the crop and region, so here is what the supplied evidence supports:
 **Pacific Northwest apple/pear guidance (US):**
@@ -2173,27 +2185,27 @@
 Note: these are historical source-specific IPM statements, not current product registrations, labels or local recommendations—check local labels and advisers. Pear-only organic recommendations are not transferred to apples.</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G21" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="22" ht="345" customHeight="1" s="7">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="22" ht="345" customHeight="1" s="1">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>H022</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand and found mealybugs in my apple orchard. How can I monitor them?</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>The evidence is limited. A New Zealand study (Hawke's Bay and Nelson) found obscure mealybug sex-pheromone traps caught male mealybugs in all 11 Hawke's Bay orchards and also caught its introduced parasitoid, which simplified monitoring of both; this was a research evaluation, not a monitoring threshold. WSU notes there is no formal monitoring scheme for apple mealybug; obvious egg sacs indicate whether later control may be needed. No New Zealand action thresholds are given in the corpus. Monitoring targets, trap types and regions differ between these studies.</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>• sex-pheromone traps can monitor obscure mealybug (and also catch its parasitoid)
 • no formal monitoring scheme or established action thresholds
@@ -2201,13 +2213,13 @@
 • does not invent NZ thresholds</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>• gives a numeric NZ action threshold
 • claims mealybugs cannot be monitored</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>The evidence does not directly address New Zealand, and its monitoring guidance comes from the Pacific Northwest (United States), so it may not apply to your conditions. Note also that it is a December 2007 technical guide.
 What the evidence says about monitoring:
@@ -2221,27 +2233,27 @@
 Gaps: the evidence gives no New Zealand-specific timing, thresholds, or sampling method, and its phenology (e.g., egg-laying in early May, hatch in early June) refers to central Washington. For a New Zealand-specific monitoring protocol, consult your local horticultural adviser, regional extension service, or plant protection authority, who can also confirm the species and any local reporting requirements.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G22" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="23" ht="358.8" customHeight="1" s="7">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="23" ht="358.8" customHeight="1" s="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>H009</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>I'm in Hawke's Bay, New Zealand. When is the fire blight risk highest and how do I know when to act?</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>New Zealand guidance says outbreaks occur at blossom when temperatures exceed 16°C, with the key infection period around flowering. A Hawke's Bay, Nelson and Waikato study (1993–1995, MARYBLYT model on Royal Gala) found few mid-bloom infection events; most predicted events were near the end of flowering or after petal fall, so secondary blooms (common on Royal Gala and Braeburn) are the main risk and early-bloom streptomycin sprays were often not aligned with infection periods. Use a risk model with weather data (a fire blight model is available through Pipfruit NZ) together with open flowers, inoculum and orchard history, and keep monitoring and removing strikes.</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>• risk is highest during blossom when temperatures exceed about 16°C
 • most infection events occur in late bloom/after petal fall; secondary blooms are at risk
@@ -2249,13 +2261,13 @@
 • monitor and remove strikes</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>• recommends routine early-bloom sprays regardless of risk
 • presents US temperature thresholds as NZ guidance</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>In Hawke's Bay, fire blight (Erwinia amylovora) risk is driven mainly by warm, wet spring weather during bloom, and the highest-risk period is flowering (especially the main bloom of susceptible cultivars) when open blossoms provide infection courts and rain, dew or high humidity allow bacteria to multiply and spread. Warm temperatures (roughly 18–24°C and above) combined with wetting events raise risk sharply; prolonged cool wet weather is less favourable. Secondary risk continues into shoot growth, especially after hail or strong wind, and on susceptible young tissue.
 To know when to act, use local decision support rather than a fixed calendar date:
@@ -2266,27 +2278,27 @@
 Act on model-flagged high-risk bloom days in consultation with your local adviser or industry body (e.g. NZ Apples and Pears / regional extension), and check current local labels and permissions for any product before use—I can't confirm current registrations or rates. Note that Hawke's Bay's specific risk timing varies with cultivar and season, so local monitoring matters more than a general date.</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="24" ht="386.4" customHeight="1" s="7">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="24" ht="386.4" customHeight="1" s="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>H012</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>My apple leaves have winding or blotchy mines inside them. What is causing this and does it need treatment?</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>These are leafminer larvae feeding inside the leaf: early (sap-feeding) larvae make snake-like mines visible from the underside, later tissue-feeding larvae make tent-like blotch mines and the upper leaf surface looks light and spotted. Low populations occur in most orchards and are usually kept down by parasitic wasps; they become pests mainly when broad-spectrum sprays disrupt these parasites. Treatment depends on mine counts and parasitism: UC IPM treats only when leaves average more than five mines per leaf, or when parasitism is low; WSU found no fruit impact below about two tissue-feeding mines per leaf in the second generation. Penn State notes apple leafminer has not caused economic injury.</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>• identifies leafminer mines
 • usually controlled by parasitoids; outbreaks follow broad-spectrum sprays
@@ -2294,13 +2306,13 @@
 • often no treatment needed</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>• recommends routine spraying for any mines
 • identifies the damage as a disease</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>**Causes**
 Winding or blotchy mines inside apple leaves are typically caused by the larvae of leaf-mining insects feeding between the upper and lower leaf surfaces. Common causes include:
@@ -2314,27 +2326,27 @@
 *Note on Pesticides:* If you consider chemical control, pesticide products, application rates, and timings vary by region and are subject to local regulatory authorization. Check your local pesticide labels and consult a local agricultural extension service or certified adviser before applying any treatments.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="25" ht="358.8" customHeight="1" s="7">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="25" ht="358.8" customHeight="1" s="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>H034</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Some leaves and young apples have dark olive-green, velvety spots, and some fruit are cracking. What is this and what should I do?</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>This is apple scab (Venturia inaequalis): velvety olive-green to black spots on leaves and fruit; fruit spots become scab-like and corky, and fruit may crack and become misshapen; badly infected leaves can yellow and drop. The fungus overwinters in fallen infected leaves, and spring rains release spores that infect young leaves and fruit. Management aims to prevent primary spring infections: reduce leaf litter (shred with a flail mower or remove it; urea on leaves before or after leaf fall speeds decomposition), prune for air movement and drying, and apply protective fungicides with exact timing and full coverage during wet periods from green tip.</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>• identifies apple scab
 • olive-green to black velvety spots; fruit spots become scabby/corky and can crack
@@ -2342,13 +2354,13 @@
 • reduce leaf litter, prune for drying, timed protective fungicides in wet periods</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>• diagnoses powdery mildew or sooty blotch
 • recommends only summer treatment and ignores primary spring infection</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Based on the symptom description, this is most consistent with **apple scab**.
 **Why:** Apple scab first appears as superficial, velvety dark-olive-to-black spots on fruit and leaves; fruit spots become scablike with age and tissues may become misshapen. The lighter-green areas that turn olive-green with fuzzy margins (spore production), plus distorted leaves and cracked/deformed fruit, also fit apple scab.
@@ -2361,27 +2373,27 @@
 **Caveats:** The treatment statements above are historical source information, not current product recommendations or proof of local authorization—check local labels and an adviser. The sources do not specify a cultivar or trial year for this guidance. If symptoms differ (e.g., purple-margined leaf spots, rusty-orange spots, or superficial soot-like patches), other diseases such as Marssonina blotch, rust, or sooty blotch/flyspeck should be considered.</t>
         </is>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="G25" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="26" ht="409.5" customHeight="1" s="7">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="26" ht="409.5" customHeight="1" s="1">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>H060</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>The shoot tips of my apple trees are covered with green aphids and the leaves are sticky with black mould. What should I do?</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>These are green aphids (green apple aphid, or the spirea aphid that has largely replaced it in some regions; they are managed together). They infest succulent terminal growth and their honeydew supports black sooty mould that hinders leaf function and lowers fruit grade; high populations on young trees can retard growth. Natural enemies (lady beetles, lacewings, syrphid fly larvae) often control them. UC IPM: a delayed dormant oil spray prevents early injury; in summer, assess predators if more than 45% of shoots are infested and consider treatment at 60% or more of terminals. Penn State: from early June sample 10 shoots on five trees and treat if more than 4.2 leaves per shoot are infested and fewer than 20% of colonies have predators.</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>• identifies green apple/spirea aphids and honeydew with sooty mould
 • natural enemies often control them
@@ -2389,13 +2401,13 @@
 • delayed dormant oil prevents early injury</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>• recommends spraying immediately regardless of predators
 • identifies them as woolly apple aphid</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Based on the supplied evidence, here's what applies to your situation:
 **What you're likely seeing**
@@ -2413,27 +2425,27 @@
 - Note: the apple grain aphid (also dark green, early-season, on buds) does little damage to apples and can even support early predator build-up — but distinguishing species rests on early appearance, bud location, and a dark green body stripe, so confirm identification rather than assume.</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n">
+      <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="27" ht="110.4" customHeight="1" s="7">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="27" ht="110.4" customHeight="1" s="1">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>H029</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Some apple leaves have small blisters that started green or red and are turning brown or black. What is it?</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>This fits blister mites (appleleaf/pearleaf blister mite): their feeding forms small galls or blisters up to about 3 mm that are green or red at first and turn light brown to black; mites live inside the leaf blisters, and fruit damaged before bloom is scarred or deformed. They are now rare in well-managed orchards and mostly attack abandoned or neglected ones. When needed, the best timing is after harvest when mites move from leaves into buds, or pre-bloom to protect fruit; summer sprays are too late to prevent fruit damage.</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>• identifies blister mites
 • green/red blisters turning brown-black; fruit scarring
@@ -2441,38 +2453,38 @@
 • post-harvest or pre-bloom timing; summer too late</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>• diagnoses a fungal leaf spot
 • recommends summer sprays to prevent fruit damage</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Based on technical guidance for the United States Pacific Northwest, small galls or blisters on foliage that are green or red at first and turn light brown to black as the tissue dies are caused by blister mites (pearleaf and appleleaf blister mite).</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n">
+      <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="28" ht="317.4" customHeight="1" s="7">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="28" ht="317.4" customHeight="1" s="1">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>H043</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Big holes have been chewed into my young apples in spring by green caterpillars. What are they?</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>These are likely green fruitworms: green caterpillars that feed on buds, flowers, leaves and young fruit in spring, often hiding in leaves webbed together on fruiting spurs; there is one generation a year. Fruittree leafroller larvae (green with a black head) can cause similar fruit damage. Fruitworm populations are patchy and can cause severe damage quickly, so sample fruit clusters from tight cluster until 2–3 weeks after petal fall. Insecticides used against codling moth appear to control green fruitworms, and Bt may give some control.</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>• identifies green fruitworm
 • spring feeding on buds, flowers and young fruit; one generation
@@ -2480,12 +2492,12 @@
 • sample clusters early; codling moth sprays or Bt</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>• identifies the caterpillars as codling moth larvae</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>I can't identify the caterpillars with certainty from your description, and the evidence supplied does not include a source describing green caterpillars chewing large holes in spring apples. The closest matches in the evidence are:
 - **Leafrollers**: Young larvae chew small pin-hole feeding sites on fruit, which are hard to see at harvest and can be mistaken for codling moth damage. Leafroller larvae are commonly found in the upper half of large trees, and spur varieties tend to show more fruit damage.
@@ -2495,27 +2507,27 @@
 Evidence is insufficient to say which species is responsible. To identify them, I'd suggest collecting a few caterpillars and taking them, along with photos of the damage, to a local extension service, plant diagnostic lab, or orchard adviser. Many of these pests have regional differences, so local identification and any treatment decisions should be confirmed with local guidance and current product labels.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="G28" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="29" ht="372.6" customHeight="1" s="7">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="29" ht="372.6" customHeight="1" s="1">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>H013</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>The young leaves on my apple trees are tightly rolled, and I found tiny orange maggots inside. What is it and does it need control?</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>This is apple leafcurling midge: larvae feed on the margins of developing leaves, which roll inward into tight tubes, may redden and later go brown and brittle. Mature trees usually do not suffer economic damage, but heavy infestations can stunt shoots of young trees and new grafts. Monitoring focuses on young trees with vigorous shoots. Insecticides are difficult because larvae are protected inside the rolls; natural enemies (e.g. the parasitoid Platygaster demades) can give useful control, and New Zealand guidance advises avoiding broad-spectrum insecticides that disrupt them.</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>• identifies apple leafcurling midge
 • tightly rolled leaves with orange larvae
@@ -2523,13 +2535,13 @@
 • natural enemies; avoid broad-spectrum sprays; larvae protected in rolls</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>• identifies the maggots as apple maggot
 • recommends routine sprays on mature trees</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Based on the description (tightly rolled young leaves containing tiny orange maggots), this is consistent with apple leaf-curling midge (Dasineura mali). Larvae are tiny legless maggots, initially pale-yellow but becoming reddish-orange as they develop inside rolled leaves, and are 1.5 to 2.5 mm long when full grown. Larvae feed on the upper leaf surface, causing the margins to roll inward. Note that the New Zealand guidance describes maggots as white or orange/pink/red, often in a cemented cocoon, but I cannot confirm species from the description alone.
 Whether it needs control depends on tree age and damage level:
@@ -2540,27 +2552,27 @@
 For a decision, check the age of your trees and how much damage is present, and consult your local horticultural adviser or extension service about current, legally registered options in your country. The evidence provided does not include New Zealand-specific thresholds or current recommendations.</t>
         </is>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G29" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="30" ht="179.4" customHeight="1" s="7">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="30" ht="179.4" customHeight="1" s="1">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>H019</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. How should I prune out European canker in my orchard?</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>New Zealand guidance: remove all visible cankers during winter pruning; because infected wood can extend beyond the visible canker, cut at least 300 mm below the lowest canker; scraping may not remove all infection; do not prune in rain; sometimes a whole limb or tree must go. Sterilise pruning tools between trees if infection is evident, and remove and burn infected material. Infection can occur all year wherever wounds exist; a New Zealand study found pruning cuts very susceptible and fruit picking and thinning wounds the most important natural entry sites, so inspect spurs (wilting leaves next to picking wounds can signal infection).</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>• remove all visible cankers in winter pruning
 • cut at least 300 mm below the lowest canker; don't prune in rain
@@ -2568,13 +2580,13 @@
 • wounds (pruning, picking, thinning, leaf scars) are infection sites; infection year-round</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>• recommends scraping cankers as sufficient
 • recommends pruning during rain</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Based on undated legacy technical guidance for New Zealand apple orchards:
 * **Timing and Conditions:** Remove all visible cankers during winter pruning. Do not prune during rain. European canker management is a season-long process, so you and your staff should be able to identify symptoms and recognize early-stage cankers.
@@ -2583,27 +2595,27 @@
 *Disclaimer: Check local labels and advisers regarding current recommendations and regulations.*</t>
         </is>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="G30" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="31" ht="151.8" customHeight="1" s="7">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="31" ht="151.8" customHeight="1" s="1">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>H024</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>My stored apples have a spongy rot that turns black, with brown-black specks around the lenticels. What could it be?</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>This fits speck rot (Phacidiopycnis washingtonensis), an emerging storage rot of apples in the US Pacific Northwest: the decay is spongy and water-soaked at first, turns brown then black while the margin stays water-soaked, and forms brown to black specks around lenticels, especially on red cultivars. It can be mistaken for gray mold, but gray mold flesh is brown whereas the speck rot margin looks translucent and water-soaked. Infection happens in the orchard (mainly stem and calyx ends, more after rain before harvest); inoculum comes mainly from crabapple pollinizers, so prune and treat pollinizers; preharvest and postharvest fungicides help (WSU).</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>• identifies speck rot (Phacidiopycnis)
 • spongy rot turning black; specks at lenticels
@@ -2611,13 +2623,13 @@
 • orchard infection; crabapple pollinizers as inoculum; fungicides</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>• diagnoses blue mold
 • says infection happens only in storage</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Based on the symptoms provided, your apples may have **speck rot** (also known as Phacidiopycnis rot, caused by *Phacidiopycnis washingtonensis*),. 
 Key symptoms of speck rot described in US Pacific Northwest technical guidance (dated April 2020) include:
@@ -2626,27 +2638,27 @@
 * In early stages, it is slightly firmer than gray mold and can be misdiagnosed as gray mold or Sphaeropsis rot,.</t>
         </is>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="32" ht="276" customHeight="1" s="7">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="32" ht="276" customHeight="1" s="1">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>H038</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>How do I know if my apple trees have woolly apple aphid on the roots?</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Root colonies are the most damaging and are found by looking at the roots and the crown just above them: roots develop large abnormal swellings (galls) and many short fibrous roots, and colonies with shorter whitish wax may be visible on roots and underground parts of the trunk. Above ground, infested trees may have yellowish foliage and young trees uproot easily. The aphid overwinters as nymphs on roots, which move up the trunk in spring and summer to start above-ground colonies.</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>• inspect roots and crown for galls/swellings and waxy colonies
 • signs: abnormal root swellings, fibrous roots, yellowish foliage, easily uprooted young trees
@@ -2654,12 +2666,12 @@
 • overwinters on roots and moves up the trunk</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>• says woolly apple aphid only lives on branches</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Based on the provided sources, you can identify a woolly apple aphid infestation on apple tree roots by checking for the following signs:
 * **Abnormal root growth:** Infested roots feature galls, swollen enlargements, or large knots,.
@@ -2672,27 +2684,27 @@
 Note that aerial (aboveground) infestations do not reliably indicate root infestations, as trees can host aerial colonies without their roots becoming infested.</t>
         </is>
       </c>
-      <c r="G32" s="6" t="n">
+      <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="33" ht="409.5" customHeight="1" s="7">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="33" ht="409.5" customHeight="1" s="1">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>H004</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Should I protect the lady beetles and predatory mites in my orchard, and how?</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Yes. Predatory mites such as Typhlodromus pyri can keep pest mites at very low levels if they are not disrupted; the mite-eating lady beetle Stethorus helps against high mite populations but arrives late and cannot be relied on alone. Avoid sprays toxic to predators: a single pyrethroid can kill beneficial mites and stimulate red mites, and some other insecticides can cause mite flare-ups; time unavoidable sprays when predators can recover. Moderate apple rust mite populations are worth keeping as food for predators. Predatory mites can be introduced on spur leaves from orchards that have them (Penn State: May to June).</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>• yes: predatory mites keep pest mites low
 • lady beetles (Stethorus) help but are not reliable alone
@@ -2700,13 +2712,13 @@
 • keep moderate rust mites as food; introduce predators on spur leaves</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>• recommends broad-spectrum sprays as compatible with predators
 • says predators are not useful</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Yes, the evidence supports conserving predatory mites as the core of apple mite management, with lady beetles playing a secondary role.
 **Why protect predatory mites:**
@@ -2726,40 +2738,40 @@
 **Limitations:** The evidence does not give current product names or label rates, and it does not specify which predators occur in your orchard or your region's current mite thresholds. Check local extension recommendations and product labels before making any treatment decisions.</t>
         </is>
       </c>
-      <c r="G33" s="6" t="n">
+      <c r="G33" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="34" ht="331.2" customHeight="1" s="7">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="34" ht="331.2" customHeight="1" s="1">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>H049</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand and some apple leaves have pale mosaic patterns. Is this apple mosaic virus and how is it managed?</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>A description of pale mosaic patterns alone cannot confirm apple mosaic virus: several causes can produce similar leaf patterns, and confirmation needs testing or expert diagnosis. The reviewed corpus contains no information on apple mosaic virus, so no evidence-based management can be given; a good answer stays cautious, does not present general advice as verified New Zealand guidance, and suggests local expert diagnosis.</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>• does not confirm apple mosaic virus from the description alone (suggests testing or expert diagnosis)
 • notes that other causes can produce similar leaf patterns
 • does not present management advice as verified New Zealand guidance</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>• confirms apple mosaic virus definitively from the description
 • attributes the patterns to another pest without any caveat</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Yes, pale yellow or cream mosaic patterns, spots, or bands on apple leaves are characteristic symptoms of Apple mosaic virus (ApMV), which is present in New Zealand. However, similar symptoms can occasionally be caused by other factors, so laboratory testing (such as ELISA or PCR) is required to confirm the diagnosis definitively.
 **Management of Apple Mosaic Virus:**
@@ -2770,27 +2782,27 @@
 * **Local Regulations:** Check current local biosecurity guidelines, registered practices, and consult a local horticulture adviser or diagnostic laboratory in New Zealand to confirm the virus and determine the best action for your specific orchard or garden setup.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="n">
+      <c r="G34" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="35" ht="386.4" customHeight="1" s="7">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="35" ht="386.4" customHeight="1" s="1">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>H028</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. My apple leaves have small dark spots and I've heard about Elsinoe leaf spot. Could that be it, and what works against it?</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>The corpus cannot confirm the diagnosis: it has no description of Elsinoe leaf spot symptoms on apple. The only Elsinoe evidence is a New Zealand glasshouse study (2009) on Royal Gala testing products suitable for organic orchards against Elsinoe piri: lime sulphur, copper hydroxide, sulphur, a low concentration of potassium carbonate and a low concentration of a Yucca schidigera extract reduced disease, while higher potassium carbonate (1%) increased severity. These are glasshouse results, not field recommendations. Other leaf-spot diseases in the corpus (e.g. apple scab, frogeye leaf spot) look different and should be considered.</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>• does not confirm Elsinoe leaf spot from the description alone
 • glasshouse tests: lime sulphur, copper, sulphur and low-rate potassium carbonate reduced disease; 1% potassium carbonate increased severity
@@ -2798,40 +2810,40 @@
 • considers other leaf-spot causes</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>• confirms Elsinoe leaf spot from the description
 • presents glasshouse results as field-proven</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>**Could it be Elsinoe leaf spot?** The evidence doesn't let us confirm that from your description alone. We have New Zealand evidence on Elsinoe leaf spot control, but the supplied excerpts do not give the symptom description for Elsinoe on apple. Small dark spots on apple leaves are also consistent with other diseases: Marssonina blotch (small grayish-brown to black spots with purple margins, mainly on mature leaves from mid-June, in Pennsylvania) and apple scab (superficial velvety dark-olive-to-black spots, California) — note these descriptions come from other regions, so they are not local diagnostic confirmation. You would need local diagnostic confirmation (e.g., your adviser or a plant pathology lab) to know what is affecting your trees.
 **What the evidence shows against Elsinoe leaf spot:** Only glasshouse/laboratory work on Royal Gala in New Zealand (2009 poster abstract) is available, and it is explicitly not a field recommendation. In those pretreatment experiments, disease incidence and severity were significantly reduced by lime sulphur (1% and 2%), low-concentration Yucca schidigera extract products (2.5%), copper hydroxide (0.009% and 0.019% copper), sulphur (0.16%), and low-concentration potassium carbonate (0.5%), compared with the control. A different saponin product, and high concentrations of potassium carbonate (1%) and a Y. schidigera product (5%), did not reduce disease; 1% potassium carbonate significantly increased severity. In laboratory tests, increasing concentrations of potassium carbonate and Y. schidigera extract reduced conidium germination and germ-tube size. These are glasshouse/lab results, not proven field treatments, and the trial years are not established from the excerpts.
 **What's missing:** There is no New Zealand field-trial evidence in these items on Elsinoe control in orchard apples, and no apple-specific Elsinoe symptom description to help you identify it. Any product use should be checked against current local labels and with a local adviser — the rates above are historical source information, not current recommendations or proof of authorization.</t>
         </is>
       </c>
-      <c r="G35" s="6" t="n">
+      <c r="G35" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="36" ht="124.2" customHeight="1" s="7">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="36" ht="124.2" customHeight="1" s="1">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>H048</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>One of my apple trees is declining, and there is a white fan-shaped fungal growth under the bark at the base. What is it?</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>This fits Armillaria root rot (oak root fungus): infected roots have white to yellowish fan-shaped mycelial mats between bark and wood, sometimes with dark rhizomorphs on the root surface. Apple rootstocks have some resistance, but high inoculum, a virulent strain or a weakened tree can overcome it; the fungus survives on dead roots. There is no truly effective control; UC IPM suggests exposing the crown and upper roots by removing soil to 9–12 inches in spring and keeping the area dry through the season, which can stop spread into the crown.</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>• identifies Armillaria root rot
 • white fan-shaped mycelial mats under bark; rhizomorphs
@@ -2839,38 +2851,38 @@
 • expose crown and upper roots and keep dry</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>• diagnoses Phytophthora or crown gall with certainty
 • recommends a fungicide spray as a cure</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>Based on the provided evidence, there is no mention of a "white fan-shaped fungal growth under the bark at the base" of apple trees. The provided sources discuss powdery mildew overwintering in white, flattened terminal buds; apple anthracnose cankers producing cream-colored fruiting bodies (acervuli),; moldy core mycelium in fruit seed cavities; and white rot lesions/cankers, but none describe a white fan-shaped fungal growth under the bark.</t>
         </is>
       </c>
-      <c r="G36" s="6" t="n">
+      <c r="G36" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="37" ht="409.5" customHeight="1" s="7">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="37" ht="409.5" customHeight="1" s="1">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>H045</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. My apple leaves have small dark spots and I've heard about Elsinoe leaf spot. Could that be it, and what works against it?</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>The corpus cannot confirm the diagnosis: it has no description of Elsinoe leaf spot symptoms on apple. The only Elsinoe evidence is a New Zealand glasshouse study (2009) on Royal Gala testing products suitable for organic orchards against Elsinoe piri: lime sulphur, copper hydroxide, sulphur, a low concentration of potassium carbonate and a low concentration of a Yucca schidigera extract reduced disease, while higher potassium carbonate (1%) increased severity. These are glasshouse results, not field recommendations. Other leaf-spot diseases in the corpus (e.g. apple scab, frogeye leaf spot) look different and should be considered.</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>• does not confirm Elsinoe leaf spot from the description alone
 • glasshouse tests: lime sulphur, copper, sulphur and low-rate potassium carbonate reduced disease; 1% potassium carbonate increased severity
@@ -2878,13 +2890,13 @@
 • considers other leaf-spot causes</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>• confirms Elsinoe leaf spot from the description
 • presents glasshouse results as field-proven</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>I can't confirm the diagnosis from a description alone, and the evidence provided does not describe Elsinoe leaf spot symptoms, so I can't say whether your spots match it.
 What the evidence does say:
@@ -2897,27 +2909,27 @@
 These are historical source results and not current label approvals. Before using any product, check the current label and local authorisation in New Zealand and consult your local orchard adviser or Plant &amp; Food Research, who can confirm the diagnosis (for example by examining lesions for the fungal structures) and recommend a current programme. The evidence provided does not include current New Zealand Elsinoe recommendations, so I cannot give one.</t>
         </is>
       </c>
-      <c r="G37" s="6" t="n">
+      <c r="G37" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="38" ht="262.2" customHeight="1" s="7">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="38" ht="262.2" customHeight="1" s="1">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>H039</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Some apples have sunken round brown spots with pinkish ooze, and the rot goes into the fruit in a cone shape. What is it?</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>This is bitter rot (Colletotrichum): sunken circular brown spots, often in concentric rings with small black dots, oozing a salmon-pink mass of spores, and a rot that progresses to the core in a V or cone shape; fruit later shrivel into mummies. It is favoured by high temperatures and humidity. Black rot differs: usually one spot per fruit and the decay is not cone-shaped. Prevention: remove dead limbs and mummified fruit (overwintering sites), keep trees vigorous, and avoid highly susceptible varieties.</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>• identifies bitter rot
 • salmon-pink spore ooze and cone/V-shaped rot
@@ -2925,13 +2937,13 @@
 • sanitation: remove mummies and dead wood; warm humid conditions favour it</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>• diagnoses bitter pit (a physiological disorder)
 • says the decay is limited to the skin</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>This description most likely points to bitter rot, caused by the fungus *Colletotrichum* (commonly *C. acutatum* or *C. gloeosporioides*). Typical features include:
 - Sunken, round, brown lesions on the fruit
@@ -2941,27 +2953,27 @@
 To confirm the diagnosis, consider a lab test or sending samples to your regional plant diagnostic service, since visual symptoms alone can be confused with other rots. Management generally involves sanitation (removing mummified fruit and cankers), pruning for airflow, and orchard-specific fungicide programs. Check your local extension service or adviser for recommended products, rates, and timings registered in your region, as these vary by location and label.</t>
         </is>
       </c>
-      <c r="G38" s="6" t="n">
+      <c r="G38" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="39" ht="331.2" customHeight="1" s="7">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="39" ht="331.2" customHeight="1" s="1">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>H008</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Part of my orchard often stays waterlogged after rain. Which apple rootstocks should I avoid there?</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Waterlogged soil favours Phytophthora root and crown rot (24 hours or more of saturated soil favours infection), so rootstock choice matters, but no rootstock is resistant to all Phytophthora species. UC IPM says MM 104 and MM 106 are generally more susceptible than M 9 and M 26. WSU rates Geneva rootstocks as most resistant, M-9 (with M-2 and M-4) as moderately susceptible, M-7 and MM-111 as moderately susceptible, M-26 and MM-106 as susceptible and MM-104 as highly susceptible; note the two sources differ on M 26. Both agree MM 104 and MM 106 are poor choices. Rootstock choice should be combined with drainage, planting on berms and avoiding standing water around crowns. These susceptibility ratings come from US sources; actual waterlogging tolerance also depends on drainage, scion and local trials.</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>• links waterlogging to Phytophthora risk
 • avoid MM 104 and MM 106
@@ -2969,13 +2981,13 @@
 • no rootstock resists all species; combine with drainage and berms</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>• recommends MM 106 or MM 104 for wet sites
 • claims a rootstock is fully resistant</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>In general, avoid rootstocks with poor tolerance of wet or poorly drained soils. The most commonly cited concerns are:
 - **Dwarfing rootstocks from the M.9 and M.26 series** (including many M.9 clones such as Nic 29 and T337). These are widely described as shallow-rooted and sensitive to waterlogging and Phytophthora root and crown rot, so they are usually the first to avoid on wet ground.
@@ -2986,27 +2998,27 @@
 If you tell me your country or region and the soil conditions, I can narrow this down further.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G39" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="40" ht="248.4" customHeight="1" s="7">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="40" ht="248.4" customHeight="1" s="1">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>H010</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Many of my apples have rough, net-like brown russeting on the skin. What could cause this?</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Several causes in the evidence produce fruit russeting. Powdery mildew can stunt and russet fruit, especially on highly susceptible cultivars. Apple rust mite feeding on the fruit skin causes tan russeting, usually concentrated around the calyx end, mainly a problem on light-coloured cultivars such as Golden Delicious. Western flower thrips feeding early in the season can leave fruit russeted at harvest (their egg-laying also causes pale pansy spots). Check for mildew on shoots in spring and for rust mites on leaves with a hand lens to narrow it down.</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>• lists more than one possible cause
 • powdery mildew can russet fruit
@@ -3014,13 +3026,13 @@
 • thrips early feeding can cause russet</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>• states a single cause with certainty
 • attributes russet to a storage rot</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Several things in the supplied evidence can cause russeting-like skin symptoms on apples, but none is confirmed as the cause of your specific "net-like" pattern:
 - **Grape mealybug honeydew** can cause a coarse, black russet scattered over the fruit surface (unlike pear psylla russeting, which is patchy/streaky), and is most common in low centers of trees. Source region: Pacific Northwest, USA.
@@ -3030,27 +3042,27 @@
 The evidence does not describe a net-like russeting pattern specifically, so I can't attribute it to a particular cause. Identification would need local diagnosis; check with your local extension adviser.</t>
         </is>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="G40" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="41" ht="179.4" customHeight="1" s="7">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="41" ht="179.4" customHeight="1" s="1">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>H026</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand and found mealybugs in my apple orchard. How can I monitor them?</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>The evidence is limited. A New Zealand study (Hawke's Bay and Nelson) found obscure mealybug sex-pheromone traps caught male mealybugs in all 11 Hawke's Bay orchards and also caught its introduced parasitoid, which simplified monitoring of both; this was a research evaluation, not a monitoring threshold. WSU notes there is no formal monitoring scheme for apple mealybug; obvious egg sacs indicate whether later control may be needed. No New Zealand action thresholds are given in the corpus. Monitoring targets, trap types and regions differ between these studies.</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>• sex-pheromone traps can monitor obscure mealybug (and also catch its parasitoid)
 • no formal monitoring scheme or established action thresholds
@@ -3058,40 +3070,40 @@
 • does not invent NZ thresholds</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>• gives a numeric NZ action threshold
 • claims mealybugs cannot be monitored</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Based on evidence from New Zealand apple orchards, obscure mealybug (*Pseudococcus viburni*) can be monitored using traps baited with obscure mealybug sex pheromone. In field evaluations, these sex pheromone traps caught male *P. viburni*. 
 Additionally, the traps serendipitously attract the parasitoid *Pseudaphycus maculipennis*, which recognizes the mealybug female sex pheromone as a kairomone. This allows the traps to simplify monitoring for the post-introduction establishment of this biological control agent alongside the mealybug.
 *(Note: In the US Pacific Northwest, technical guidance notes there are no formal schemes for monitoring apple mealybug (*Phenacoccus aceris*), though their egg sacs become apparent when abundant.)*</t>
         </is>
       </c>
-      <c r="G41" s="6" t="n">
+      <c r="G41" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="42" ht="409.5" customHeight="1" s="7">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="42" ht="409.5" customHeight="1" s="1">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>H050</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. How should I prune out European canker in my orchard?</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>New Zealand guidance: remove all visible cankers during winter pruning; because infected wood can extend beyond the visible canker, cut at least 300 mm below the lowest canker; scraping may not remove all infection; do not prune in rain; sometimes a whole limb or tree must go. Sterilise pruning tools between trees if infection is evident, and remove and burn infected material. Infection can occur all year wherever wounds exist; a New Zealand study found pruning cuts very susceptible and fruit picking and thinning wounds the most important natural entry sites, so inspect spurs (wilting leaves next to picking wounds can signal infection).</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>• remove all visible cankers in winter pruning
 • cut at least 300 mm below the lowest canker; don't prune in rain
@@ -3099,13 +3111,13 @@
 • wounds (pruning, picking, thinning, leaf scars) are infection sites; infection year-round</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>• recommends scraping cankers as sufficient
 • recommends pruning during rain</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>European canker (Neonectria ditissima) is a serious issue in New Zealand apple orchards. General approach to pruning it out:
 **Timing**
@@ -3125,27 +3137,27 @@
 For region-specific timing and any registered wound-treatment options, confirm with your local adviser, since NZ conditions and label approvals change.</t>
         </is>
       </c>
-      <c r="G42" s="6" t="n">
+      <c r="G42" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="43" ht="409.5" customHeight="1" s="7">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="43" ht="409.5" customHeight="1" s="1">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>H031</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>How should I time my sprays for codling moth?</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Sprays target hatching larvae, so timing comes from pheromone traps plus degree-days. Set a biofix from the first sustained moth catch (UC IPM: moths in traps for three consecutive checks and sunset temperature at least 62°F; Penn State: first capture), then accumulate degree-days (base 50°F, upper 88°F). UC IPM sprays at about 250 degree-days after biofix (160 if catches are high), repeating when residual ends; Penn State applies at 250–350 degree-days, or within 5–8 days when catches exceed five moths per trap per week without mating disruption. Two to four generations occur per year, so track each generation and check fruit for damage. These biofix rules, degree-day values and thresholds come from US programmes (California, Pennsylvania); local models, product labels and conditions determine actual timing.</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>• sprays target egg hatch/young larvae
 • pheromone traps to set a biofix
@@ -3153,13 +3165,13 @@
 • multiple generations; repeat timing and fruit checks</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>• recommends calendar sprays without monitoring
 • presents one region's threshold as universal</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t># Timing codling moth sprays
 Timing depends on your region and monitoring setup, so the two sources below give different schemes and should not be mixed.
@@ -3178,27 +3190,27 @@
 In short: use pheromone traps to set biofix and monitor, then accumulate degree-days (base 50°F) and follow your local region's thresholds. These are historical source guidelines, not current label recommendations — check local labels and advisers before choosing products, rates or timings.</t>
         </is>
       </c>
-      <c r="G43" s="6" t="n">
+      <c r="G43" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="44" ht="409.5" customHeight="1" s="7">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="44" ht="409.5" customHeight="1" s="1">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>H014</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. My apple leaves have small dark spots and I've heard about Elsinoe leaf spot. Could that be it, and what works against it?</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>The corpus cannot confirm the diagnosis: it has no description of Elsinoe leaf spot symptoms on apple. The only Elsinoe evidence is a New Zealand glasshouse study (2009) on Royal Gala testing products suitable for organic orchards against Elsinoe piri: lime sulphur, copper hydroxide, sulphur, a low concentration of potassium carbonate and a low concentration of a Yucca schidigera extract reduced disease, while higher potassium carbonate (1%) increased severity. These are glasshouse results, not field recommendations. Other leaf-spot diseases in the corpus (e.g. apple scab, frogeye leaf spot) look different and should be considered.</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>• does not confirm Elsinoe leaf spot from the description alone
 • glasshouse tests: lime sulphur, copper, sulphur and low-rate potassium carbonate reduced disease; 1% potassium carbonate increased severity
@@ -3206,13 +3218,13 @@
 • considers other leaf-spot causes</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>• confirms Elsinoe leaf spot from the description
 • presents glasshouse results as field-proven</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Based on New Zealand research using 'Royal Gala' glasshouse seedlings and laboratory experiments, treatments tested against *Elsinoe leaf spot* (*Elsinoe piri*) produced the following results:
 * **Treatments that significantly reduced disease incidence and severity:**
@@ -3232,27 +3244,27 @@
 * Pesticide efficacy, registration, and product rates vary by region and date. Always check current local pesticide labels and consult a local orchard advisor before applying treatments.</t>
         </is>
       </c>
-      <c r="G44" s="6" t="n">
+      <c r="G44" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="45" ht="409.5" customHeight="1" s="7">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="45" ht="409.5" customHeight="1" s="1">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>H052</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Some branches have sunken cankers with rings around buds and leaf scars, and the bark is flaky in the centre. What is it?</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>This fits European canker (Neonectria ditissima): it starts as small dark sunken areas around buds, leaf scars or wounds, which develop concentric rings of cracking with swelling of the stem above and below, a dry flaky centre and staining of the wood beneath; white spores form in the cracks in humid weather and dark red fruiting bodies in autumn and winter. Flaky bark alone is not unique to this disease. The fungus enters through leaf scars, growth cracks and wounds, and cankers kill branches; infected wood should be pruned out well below the canker and destroyed.</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>• identifies European canker
 • sunken areas at buds/leaf scars with concentric rings; white spores or red fruiting bodies
@@ -3260,13 +3272,13 @@
 • prune out infected wood below the canker and destroy it</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>• diagnoses fire blight without considering the ring pattern
 • says the canker will heal by itself</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Based on the symptoms described, the most likely cause is European canker (caused by *Nectria galligena*, the fungus associated with this disease in the supplied New Zealand sources). Sunken cankers with concentric rings that begin at buds, leaf scars, or wounds, and that dry out and become flaky in the centre, match the initial and progressive symptoms described in the New Zealand guidance. Concentric cracking and blackened, sunken bark are also described for European canker on apple.
 Points that support this identification and points that limit it:
@@ -3277,27 +3289,27 @@
 Management: the supplied sources give cultural sanitation and pruning measures as relevant options, but they do not provide current, locally authorised pesticide recommendations. Please consult your regional extension service or a local horticultural adviser for diagnosis confirmation and for any control measures or product labels that apply where you are.</t>
         </is>
       </c>
-      <c r="G45" s="6" t="n">
+      <c r="G45" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="46" ht="372.6" customHeight="1" s="7">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="46" ht="372.6" customHeight="1" s="1">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>H002</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>In winter I see dark, sunken, cracked patches on some branches of my apple trees. What could they be?</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Several canker diseases produce this, so look closely before deciding. Fire blight overwintering cankers can be black, grey, violet or brown with dry sunken tissue, and reddish flecking under the bark at the edge of an active canker. European canker starts as small sunken areas at leaf scars, buds or wounds and develops concentric rings of cracking with swelling of the stem around it. Apple anthracnose cankers are elongated, sunken, orange to brown, with cracking around the margin. Black rot cankers are reddish brown and slightly sunken, sometimes expanding each year. In all cases cankers are inoculum sources, so the general response is to prune out cankered wood well into healthy tissue and destroy it.</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>• recognises several canker causes rather than one definite diagnosis
 • gives at least two distinguishing features (e.g. concentric rings at leaf scars for European canker; reddish flecking at margin for fire blight; orange-brown elongated for anthracnose)
@@ -3305,13 +3317,13 @@
 • prune out cankered wood into healthy tissue and destroy it</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>• gives a single definitive diagnosis without distinguishing features
 • says cankers can be left because they are harmless</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>Dark, sunken, and cracked patches on apple tree branches seen in winter are typical symptoms of **cankers**. 
 In apples, these are most commonly caused by fungal or bacterial pathogens. The most frequent causes include:
@@ -3324,27 +3336,27 @@
 **Note:** Physical identification depends on your specific region, tree cultivar, and microclimate. For accurate diagnosis and localized control guidance, consult a local agricultural extension officer or certified arborist, and check local labels before applying any protective chemical treatments.</t>
         </is>
       </c>
-      <c r="G46" s="6" t="n">
+      <c r="G46" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="47" ht="409.5" customHeight="1" s="7">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="47" ht="409.5" customHeight="1" s="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>H041</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>What can I do to reduce apple scab next year?</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Focus on reducing overwintering spores and preventing spring infections. The fungus overwinters on fallen infected leaves, so shred them with a flail mower or remove them; urea applied to leaves before leaf fall or on fallen leaves reduces ascospores by 50–75% (Canadian crop profile). Prune for air movement and drying, avoid excess nitrogen that produces susceptible suckers, plant scab-resistant cultivars, and do not leave fruit on the ground. Time protective fungicides to spring infection periods with full coverage, using wetness and temperature prediction tools; if primary infections are controlled, secondary infections will not be serious.</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>• remove or shred fallen leaves; urea speeds decomposition
 • pruning for drying; avoid excess nitrogen; resistant cultivars
@@ -3352,13 +3364,13 @@
 • controlling primary infections prevents serious secondary infection</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>• recommends only summer fungicides
 • says leaf litter is irrelevant</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>To reduce apple scab (Venturia inaequalis) next year, focus on lowering overwintering inoculum and protecting new growth in spring. Key measures:
 **Winter/early spring (before bud break)**
@@ -3379,27 +3391,27 @@
 For cultivar-specific or organic options, local extension guidance for your region is the best next step.</t>
         </is>
       </c>
-      <c r="G47" s="6" t="n">
+      <c r="G47" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="48" ht="124.2" customHeight="1" s="7">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="48" ht="124.2" customHeight="1" s="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>H001</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>My apple leaves have lots of tiny white speckles, and small pale insects jump off when I touch the leaves. What are they?</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>These are leafhoppers, most likely white apple leafhopper (rose leafhopper looks almost identical). Their feeding causes white or yellowish-white stippling; unlike mite feeding the spots are larger and there is no bronzing. Excrement leaves black specks on fruit that wash off, and adults are a nuisance to pickers at harvest. In Washington no fruit size or quality effect was found even at high populations. UC IPM: monitor from petal fall and treat first-generation nymphs only above about 0.5 nymphs per leaf or 30% infested leaves.</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>• identifies leafhoppers (white apple leafhopper)
 • white stippling without bronzing distinguishes from mites
@@ -3407,39 +3419,39 @@
 • threshold-based nymph treatment (e.g. 0.5 nymphs/leaf)</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>• identifies the insects as aphids or mites
 • claims leafhoppers cause major fruit loss in all cases</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>Based on the provided evidence, leafhoppers cause white stippling, speckling, or mottling on apple leaves by sucking sap from leaf tissue,,. Leafhopper adults and nymphs feed on the leaves,; the adults are white, and the nymphs are whitish or whitish-green,. 
 The exact species cannot be confirmed from the physical description alone, as the provided sources specify regional traits for the white apple leafhopper (*Typhlocyba pomaria*),,, and general leafhoppers.</t>
         </is>
       </c>
-      <c r="G48" s="6" t="n">
+      <c r="G48" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="49" ht="409.5" customHeight="1" s="7">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="49" ht="409.5" customHeight="1" s="1">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>H021</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>How do I put out pheromone dispensers to control codling moth?</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Hang hand-applied dispensers in the upper third of the canopy shortly before the first moth emergence (UC IPM uses historical biofix dates; early to avoid late mating), and reapply according to the product's life if it will not last through the season. Puffers go inside edge trees or outside second-row trees at about 20 units per quarter mile. Mating disruption works best in large, uniform, square blocks (not under about 3–5 acres per UC IPM; WSU notes small orchards under 10 acres or near pest sources may not get reliable control). In the first year or with moderate to high populations, supplementary insecticides are usually needed; keep monitoring traps (high-load lures) and fruit. Dispenser rates and placement follow the product label and local registration; the UC IPM figures are not universal.</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>• place dispensers in upper canopy before first moth flight
 • best in large uniform blocks; small/isolated issues
@@ -3447,13 +3459,13 @@
 • keep monitoring with traps and fruit checks</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>• says pheromones kill moths
 • recommends mating disruption alone for high populations</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>**Short answer:** Hang pheromone dispensers (for mating disruption) throughout the orchard before the first moths emerge in spring, at the labeled density per hectare, distributed evenly and at the labeled height in the upper canopy. Specific product, rate, and timing vary by product and country — check the local label and a local adviser.
 **Key points (general, across regions):**
@@ -3466,27 +3478,27 @@
 **Caveats:** Product rates, dispenser heights, and timing are product- and country-specific, and label approval varies. This is general guidance, not a current recommendation for your area — confirm with your local label and extension adviser.</t>
         </is>
       </c>
-      <c r="G49" s="6" t="n">
+      <c r="G49" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="50" ht="248.4" customHeight="1" s="7">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="50" ht="248.4" customHeight="1" s="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>H057</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>My stored apples have a spongy rot that turns black, with brown-black specks around the lenticels. What could it be?</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>This fits speck rot (Phacidiopycnis washingtonensis), an emerging storage rot of apples in the US Pacific Northwest: the decay is spongy and water-soaked at first, turns brown then black while the margin stays water-soaked, and forms brown to black specks around lenticels, especially on red cultivars. It can be mistaken for gray mold, but gray mold flesh is brown whereas the speck rot margin looks translucent and water-soaked. Infection happens in the orchard (mainly stem and calyx ends, more after rain before harvest); inoculum comes mainly from crabapple pollinizers, so prune and treat pollinizers; preharvest and postharvest fungicides help (WSU).</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>• identifies speck rot (Phacidiopycnis)
 • spongy rot turning black; specks at lenticels
@@ -3494,13 +3506,13 @@
 • orchard infection; crabapple pollinizers as inoculum; fungicides</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>• diagnoses blue mold
 • says infection happens only in storage</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>Based on the supplied evidence, this most closely matches **apple speck rot (Phacidiopycnis rot)**, caused by *Phacidiopycnis washingtonensis*.
 Key matches:
@@ -3513,27 +3525,27 @@
 - The evidence does not establish whether this occurs in your region or storage conditions; it describes symptom appearance only.</t>
         </is>
       </c>
-      <c r="G50" s="6" t="n">
+      <c r="G50" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="51" ht="331.2" customHeight="1" s="7">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="51" ht="331.2" customHeight="1" s="1">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>H015</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>Small worms are feeding just under the skin of my apples, leaving shallow trails, but they don't reach the core. What could they be?</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>This fits lesser appleworm: larvae form extensive shallow mines under the fruit skin, may burrow deeper but not into the core, and in autumn often feed around the calyx. Codling moth differs because its larvae tunnel to the core. European apple sawfly's first larval stage also tunnels just under the skin, leaving a ribbon-like scar, before later larvae bore into the seed cavity. Lesser appleworm is usually not an economic pest: codling moth controls (except codling-moth-only mating disruption) also control it, and WSU says control is not necessary.</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>• identifies lesser appleworm
 • shallow mines under skin, not into core
@@ -3541,13 +3553,13 @@
 • usually not economic; codling moth programme controls it</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>• identifies the larvae as codling moth
 • recommends a dedicated spray programme</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Shallow trails just under the skin that don't reach the core usually point to larval feeding by leafrollers or similar small caterpillars, or to sap-feeding/surface-feeding pests. Common candidates on apples include:
 - **Leafroller larvae** (e.g., tortricid moths such as the obliquebanded leafroller or light brown apple moth, depending on region). They often feed on the surface and just under the skin, sometimes webbing leaves or fruit together.
@@ -3559,39 +3571,39 @@
 For any control measures, check current product labels and recommendations from your local authority or adviser, as registrations and timings vary by country.</t>
         </is>
       </c>
-      <c r="G51" s="6" t="n">
+      <c r="G51" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="52" ht="409.5" customHeight="1" s="7">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="52" ht="409.5" customHeight="1" s="1">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>H056</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Can I use insect netting to keep pests off my apple trees?</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>The corpus has only limited evidence. A Quebec study (abstract excerpt only) on insect netting found that, for a similar opening area, an elongated rectangular mesh appears to let beneficial insects through while still protecting against apple pests. The corpus does not provide practical installation, cost or pest-by-pest effectiveness guidance, so a full recommendation cannot be given from it.</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>• reports the netting study finding (rectangular mesh lets beneficials through while protecting against pests)
 • presents the mesh finding as limited research evidence, not established practice
 • notes practical installation and pest-by-pest effectiveness are uncertain or need further advice</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>• gives detailed netting specifications or claims complete pest exclusion without support</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Short answer: the supplied evidence gives only partial support for insect netting on apples, and it does not give quantified mesh specifications or confirm that netting is a complete solution.
 What the evidence supports:
@@ -3606,27 +3618,27 @@
 To decide whether netting is suitable for your orchard, check with your local horticultural extension service or adviser, who can identify your key pests and confirm locally authorised options, including the current pesticide labels for your area.</t>
         </is>
       </c>
-      <c r="G52" s="6" t="n">
+      <c r="G52" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="53" ht="386.4" customHeight="1" s="7">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="53" ht="386.4" customHeight="1" s="1">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>H058</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>The shoot tips of my apple trees are covered with green aphids and the leaves are sticky with black mould. What should I do?</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>These are green aphids (green apple aphid, or the spirea aphid that has largely replaced it in some regions; they are managed together). They infest succulent terminal growth and their honeydew supports black sooty mould that hinders leaf function and lowers fruit grade; high populations on young trees can retard growth. Natural enemies (lady beetles, lacewings, syrphid fly larvae) often control them. UC IPM: a delayed dormant oil spray prevents early injury; in summer, assess predators if more than 45% of shoots are infested and consider treatment at 60% or more of terminals. Penn State: from early June sample 10 shoots on five trees and treat if more than 4.2 leaves per shoot are infested and fewer than 20% of colonies have predators.</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>• identifies green apple/spirea aphids and honeydew with sooty mould
 • natural enemies often control them
@@ -3634,13 +3646,13 @@
 • delayed dormant oil prevents early injury</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>• recommends spraying immediately regardless of predators
 • identifies them as woolly apple aphid</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Based on the evidence, the symptoms you describe (green aphids on shoot tips, sticky leaves, black mould) match green apple aphid infestation with honeydew and sooty mould. Green aphids feed mainly on new leaves and growing shoots, and their honeydew supports black sooty mould that reduces leaf photosynthesis. Heavy honeydew and mould can hinder leaf function and lower fruit grade.
 Points to consider:
@@ -3651,27 +3663,27 @@
 The evidence provided does not include current pesticide options, rates, or timings for your region, and the sources are historical US guidance rather than advice for your location. For any chemical control decision, check current product labels and consult a local horticultural adviser or extension service, as product availability and authorization vary by country.</t>
         </is>
       </c>
-      <c r="G53" s="6" t="n">
+      <c r="G53" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="54" ht="248.4" customHeight="1" s="7">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="54" ht="248.4" customHeight="1" s="1">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>H047</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>Part of my orchard often stays waterlogged after rain. Which apple rootstocks should I avoid there?</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Waterlogged soil favours Phytophthora root and crown rot (24 hours or more of saturated soil favours infection), so rootstock choice matters, but no rootstock is resistant to all Phytophthora species. UC IPM says MM 104 and MM 106 are generally more susceptible than M 9 and M 26. WSU rates Geneva rootstocks as most resistant, M-9 (with M-2 and M-4) as moderately susceptible, M-7 and MM-111 as moderately susceptible, M-26 and MM-106 as susceptible and MM-104 as highly susceptible; note the two sources differ on M 26. Both agree MM 104 and MM 106 are poor choices. Rootstock choice should be combined with drainage, planting on berms and avoiding standing water around crowns. These susceptibility ratings come from US sources; actual waterlogging tolerance also depends on drainage, scion and local trials.</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>• links waterlogging to Phytophthora risk
 • avoid MM 104 and MM 106
@@ -3679,40 +3691,40 @@
 • no rootstock resists all species; combine with drainage and berms</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>• recommends MM 106 or MM 104 for wet sites
 • claims a rootstock is fully resistant</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>In a waterlogged spot, avoid the most Phytophthora-susceptible apple rootstocks. Based on US Pacific Northwest extension guidance, MM-104 is highly susceptible; M-26 and MM-106 are susceptible; and M-7, MM-111, M-9, M-2 and M-4 are moderately susceptible. California guidance similarly notes that MM 104 and MM 106 are generally more susceptible than M 9 and M 26. Canadian guidance lists M.26, M.7 and MM.106 among the most susceptible.
 If you want less susceptible options, the Geneva series is described as most resistant among dwarfing apple rootstocks in the Pacific Northwest source, and Canadian guidance names CG.30, CG.6210 and G.16 as resistant to crown and root rot. Note that no rootstock is resistant to all Phytophthora species, so success can depend on which species is present.
 Also address the waterlogging itself: improve drainage, avoid standing water around crowns, plant on berms, and use shorter/more frequent irrigations; saturated soil for 24 hours or more favors infection. These sources are US/Canadian guidance from their stated dates and are not local authorisation or current recommendations for your region—check local labels and advisers.</t>
         </is>
       </c>
-      <c r="G54" s="6" t="n">
+      <c r="G54" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="55" ht="400.2" customHeight="1" s="7">
-      <c r="A55" s="5" t="inlineStr">
+    <row r="55" ht="400.2" customHeight="1" s="1">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>H051</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>I'm in New Zealand. My apple leaves have small dark spots and I've heard about Elsinoe leaf spot. Could that be it, and what works against it?</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>The corpus cannot confirm the diagnosis: it has no description of Elsinoe leaf spot symptoms on apple. The only Elsinoe evidence is a New Zealand glasshouse study (2009) on Royal Gala testing products suitable for organic orchards against Elsinoe piri: lime sulphur, copper hydroxide, sulphur, a low concentration of potassium carbonate and a low concentration of a Yucca schidigera extract reduced disease, while higher potassium carbonate (1%) increased severity. These are glasshouse results, not field recommendations. Other leaf-spot diseases in the corpus (e.g. apple scab, frogeye leaf spot) look different and should be considered.</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>• does not confirm Elsinoe leaf spot from the description alone
 • glasshouse tests: lime sulphur, copper, sulphur and low-rate potassium carbonate reduced disease; 1% potassium carbonate increased severity
@@ -3720,13 +3732,13 @@
 • considers other leaf-spot causes</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>• confirms Elsinoe leaf spot from the description
 • presents glasshouse results as field-proven</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>I can't confirm a diagnosis from a description, and the evidence supplied doesn't describe Elsinoe leaf spot symptoms, so I can't say whether your spots match it. The evidence also does not include Elsinoe lesion descriptions for New Zealand field conditions.
 What the evidence does say:
@@ -3736,27 +3748,27 @@
 Practical next steps: have the leaves examined by a plant pathologist or your local orchard adviser (for example, through Plant &amp; Food Research or your regional horticulture advisory service). Confirm any product's registration and label for apples in New Zealand before use, since the products mentioned are historical research findings, not current recommendations.</t>
         </is>
       </c>
-      <c r="G55" s="6" t="n">
+      <c r="G55" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="56" ht="317.4" customHeight="1" s="7">
-      <c r="A56" s="5" t="inlineStr">
+    <row r="56" ht="317.4" customHeight="1" s="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>H007</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>How do I know if my apple trees have woolly apple aphid on the roots?</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>Root colonies are the most damaging and are found by looking at the roots and the crown just above them: roots develop large abnormal swellings (galls) and many short fibrous roots, and colonies with shorter whitish wax may be visible on roots and underground parts of the trunk. Above ground, infested trees may have yellowish foliage and young trees uproot easily. The aphid overwinters as nymphs on roots, which move up the trunk in spring and summer to start above-ground colonies.</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>• inspect roots and crown for galls/swellings and waxy colonies
 • signs: abnormal root swellings, fibrous roots, yellowish foliage, easily uprooted young trees
@@ -3764,12 +3776,12 @@
 • overwinters on roots and moves up the trunk</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>• says woolly apple aphid only lives on branches</t>
         </is>
       </c>
-      <c r="F56" s="5" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>You can't reliably tell from the top of the tree. Evidence from the Pacific Northwest states that aerial infestations are not a true indication of root infestations—trees can have aerial colonies all season without their roots becoming infested. So above-ground signs alone don't confirm root infestation.
 What to look for on the roots themselves (based on described symptoms):
@@ -3782,27 +3794,27 @@
 The supplied sources do not describe a specific scouting or root-sampling protocol (e.g., digging, timing, sample size) for confirming root infestation in apples, so that detail is missing from this evidence.</t>
         </is>
       </c>
-      <c r="G56" s="6" t="n">
+      <c r="G56" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="57" ht="409.5" customHeight="1" s="7">
-      <c r="A57" s="5" t="inlineStr">
+    <row r="57" ht="409.5" customHeight="1" s="1">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>H016</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>I'm in Nelson, New Zealand. Can parasitic wasps control woolly apple aphid in my orchard?</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Yes, with conditions. At Appleby near Nelson (1994–96), the parasitoid Aphelinus mali reached over 80% parasitism in the second season and controlled the aphid without aphicide sprays within a selective (tebufenozide-based) programme. But this biocontrol is fragile: a Hawke's Bay study linked the 2007–08 outbreaks mainly to spinetoram, which is toxic to A. mali, and noted other insecticides also contribute; with no available aphicide, avoiding disruptive sprays is essential. A. mali only parasitises above-ground colonies; look for black mummified aphids with round exit holes. WSU adds that generalist predators are also important and that control may fail after mild winters. These results come from specific trials and seasons; the same parasitism or control is not guaranteed in every Nelson orchard today.</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>• yes: A. mali controlled WAA in a Nelson trial with selective insecticides
 • disruptive insecticides (e.g. spinetoram) caused outbreaks; avoid them
@@ -3810,13 +3822,13 @@
 • predators also help; mild winters may limit control</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>• says parasitoids cannot control woolly apple aphid
 • recommends spinetoram for aphid control</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Yes, there is New Zealand evidence that the parasitic wasp *Aphelinus mali* can control woolly apple aphid in Nelson apple orchards, but with conditions.
 - In a Nelson study (1994–1996, Appleby Research Orchard), *A. mali* established and regulated woolly apple aphid populations over two seasons within an experimental Integrated Fruit Production programme that included the insect growth regulator tebufenozide. Aphid control was achieved without specific aphicide sprays. Parasitism reached 13% by the end of April 1995 in the first season and over 80% by late April 1996 in the second.
@@ -3829,27 +3841,27 @@
 Evidence is insufficient to say how reliably *A. mali* controls aphids across Nelson orchards generally, or what your current pesticide programme would do to it. Check your local pesticide labels and consult a New Zealand horticultural adviser or Plant &amp; Food Research for current, locally appropriate monitoring and management advice.</t>
         </is>
       </c>
-      <c r="G57" s="6" t="n">
+      <c r="G57" s="7" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="58" ht="220.8" customHeight="1" s="7">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="58" ht="220.8" customHeight="1" s="1">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>H055</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>My apples have dark sooty smudges and clusters of tiny black dots on the skin. What is this and is it harmful?</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>These are sooty blotch (olive-green to dark sooty patches with irregular edges) and flyspeck (clusters of small shiny black dots), two fungal diseases that usually appear together in summer. They are superficial and only on the skin, but they spoil the appearance and reduce market value. They are favoured by long periods of high humidity and rain; inoculum comes from twigs and wild hosts such as brambles in hedgerows. Prevention: prune for air movement, mow grass to lower humidity, and reduce alternate hosts around the orchard. (Leafhopper excrement also leaves black specks, but those wash off.)</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>• identifies sooty blotch and flyspeck
 • superficial skin blemish that lowers market value, not internal rot
@@ -3857,13 +3869,13 @@
 • pruning, mowing, reducing alternate hosts</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>• says the fruit is rotten inside
 • recommends discarding all fruit as unsafe</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Your apples most likely have **sooty blotch and flyspeck** — two distinct fungal diseases that commonly appear together on apple fruit in summer because they favor the same cool, humid conditions.
 - **Sooty blotch** (caused by *Gloeodes pomigena*) shows as dark brown or olive-green smudgy colonies with irregular edges, resembling soot on the fruit surface.
@@ -3872,27 +3884,27 @@
 Note this is US-based guidance; for confirmation of diagnosis and any management decisions, consult your local extension adviser.</t>
         </is>
       </c>
-      <c r="G58" s="6" t="n">
+      <c r="G58" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="59" ht="331.2" customHeight="1" s="7">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="59" ht="331.2" customHeight="1" s="1">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>H059</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>My apple leaves have winding or blotchy mines inside them. What is causing this and does it need treatment?</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>These are leafminer larvae feeding inside the leaf: early (sap-feeding) larvae make snake-like mines visible from the underside, later tissue-feeding larvae make tent-like blotch mines and the upper leaf surface looks light and spotted. Low populations occur in most orchards and are usually kept down by parasitic wasps; they become pests mainly when broad-spectrum sprays disrupt these parasites. Treatment depends on mine counts and parasitism: UC IPM treats only when leaves average more than five mines per leaf, or when parasitism is low; WSU found no fruit impact below about two tissue-feeding mines per leaf in the second generation. Penn State notes apple leafminer has not caused economic injury.</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>• identifies leafminer mines
 • usually controlled by parasitoids; outbreaks follow broad-spectrum sprays
@@ -3900,13 +3912,13 @@
 • often no treatment needed</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>• recommends routine spraying for any mines
 • identifies the damage as a disease</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>Winding or blotchy mines inside apple leaves are almost certainly caused by leafminer larvae. The most common culprits on apple are:
 - **Apple leafminer (Phyllonorycta blancardella)**: creates a silvery or whitish blotch mine on the upper leaf surface, often with a blistered or puckered appearance.
@@ -3916,27 +3928,27 @@
 If you decide to act, options include encouraging natural enemies, removing and destroying heavily mined leaves in autumn to reduce overwintering pupae, and, where needed, using an insecticide. Insecticide timing is critical because the larvae are protected inside the leaf, so products are generally aimed at the adult moths or at the early stage before tunnelling. Check your local product labels and ask a local adviser which products are authorised for apples in your area and what timing applies there, as recommendations vary by country and region.</t>
         </is>
       </c>
-      <c r="G59" s="6" t="n">
+      <c r="G59" s="7" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="60" ht="409.5" customHeight="1" s="7">
-      <c r="A60" s="5" t="inlineStr">
+    <row r="60" ht="409.5" customHeight="1" s="1">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>H020</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>My apple leaves have winding or blotchy mines inside them. What is causing this and does it need treatment?</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>These are leafminer larvae feeding inside the leaf: early (sap-feeding) larvae make snake-like mines visible from the underside, later tissue-feeding larvae make tent-like blotch mines and the upper leaf surface looks light and spotted. Low populations occur in most orchards and are usually kept down by parasitic wasps; they become pests mainly when broad-spectrum sprays disrupt these parasites. Treatment depends on mine counts and parasitism: UC IPM treats only when leaves average more than five mines per leaf, or when parasitism is low; WSU found no fruit impact below about two tissue-feeding mines per leaf in the second generation. Penn State notes apple leafminer has not caused economic injury.</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>• identifies leafminer mines
 • usually controlled by parasitoids; outbreaks follow broad-spectrum sprays
@@ -3944,13 +3956,13 @@
 • often no treatment needed</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>• recommends routine spraying for any mines
 • identifies the damage as a disease</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>Winding or blotchy mines inside apple leaves are consistent with leafminer larvae. The evidence describes two possibilities, and the sources do not allow a definite identification from your description alone.
 **Likely cause: a leafminer.** Apple leafminer larvae make a winding linear mine that widens into a blotch mine on the upper leaf surface. Frass ejected through holes in the lower epidermis often hangs from the mine in threads, and leaf tissue beyond the mine may turn chlorotic. Western tentiform leafminer also causes tissue-feeding mines on apple foliage. The two are hard to tell apart from appearance alone; apple leafminer adults resemble spotted tentiform leafminer. Inspecting the mine for frass threads and checking leaf undersides for feeding holes may help.
@@ -3962,27 +3974,27 @@
 **Missing information:** The evidence does not give current local thresholds, monitoring methods for your area, or approved control products. Before any treatment decision, count mines per leaf, check for frass and leaf-underside holes, and consult your regional extension service or a local adviser, who can confirm the species and advise on current, locally registered options.</t>
         </is>
       </c>
-      <c r="G60" s="6" t="n">
+      <c r="G60" s="7" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="61" ht="248.4" customHeight="1" s="7">
-      <c r="A61" s="5" t="inlineStr">
+    <row r="61" ht="248.4" customHeight="1" s="1">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>H025</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>There are white, mealy insects in the calyx end of my apples. What are they?</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>These may be mealybugs, such as apple mealybug, whose females have a white waxy coating (sage-green body underneath) and can be found in the apple calyx. Woolly apple aphids can also settle in the calyx when their parasite is absent, so check whether the insects are covered in long white woolly wax. For apple mealybug WSU notes there is no formal monitoring scheme; dormant or delayed dormant sprays and treatment at crawler emergence are the vulnerable points, good coverage of bark crevices matters, and parasitoids help keep it low if not disrupted by pesticides.</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>• suggests mealybugs (e.g. apple mealybug)
 • considers woolly apple aphid in the calyx as an alternative
@@ -3990,13 +4002,13 @@
 • parasitoids help; avoid disruptive pesticides</t>
         </is>
       </c>
-      <c r="E61" s="5" t="inlineStr">
+      <c r="E61" s="6" t="inlineStr">
         <is>
           <t>• identifies them as powdery mildew
 • states a firm treatment threshold that the source does not give</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>The evidence suggests they may be apple mealybugs, though the sources do not confirm an identification from your description.
 - Apple mealybug has been documented in apple calyx ends in the US Pacific Northwest; a source photo shows it in an apple calyx.
@@ -4005,7 +4017,7 @@
 The evidence does not describe control measures for apple mealybug in apples, and I cannot confirm the identification from your description alone. Please send a photo or sample to your local extension service or fruit-crop diagnostic lab, and check current local labels and advice before any treatment.</t>
         </is>
       </c>
-      <c r="G61" s="6" t="n">
+      <c r="G61" s="7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4029,90 +4041,90 @@
   <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="130" customWidth="1" style="7" min="1" max="1"/>
+    <col width="130" customWidth="1" style="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Rater: Mengshuai Feng</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Score every row 0-4 using this rubric:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>4 = Core answer (diagnosis or main fact) correct; advice complete and correct</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>3 = Core answer correct; main advice correct, only secondary details missing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2 = Core answer correct, but advice sparse or generic</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>1 = Core answer uncertain or only partly correct, but some useful correct information</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>0 = Wrong core answer, any listed major error, or no useful content</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n"/>
+      <c r="A9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n"/>
+      <c r="A10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n"/>
+      <c r="A11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n"/>
+      <c r="A12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n"/>
+      <c r="A13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n"/>
+      <c r="A14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n"/>
+      <c r="A15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n"/>
+      <c r="A16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n"/>
+      <c r="A17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n"/>
+      <c r="A18" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>